<commit_message>
Completar sitio y preparar publicación
</commit_message>
<xml_diff>
--- a/labsemco-contenido-google-sheets.xlsx
+++ b/labsemco-contenido-google-sheets.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido" sheetId="1" r:id="R93d41575bdba466b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrusel" sheetId="2" r:id="R7650580f21624acb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investigación" sheetId="3" r:id="R95998fd7d5f54d02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="4" r:id="R4cbd31f8556e4c4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="5" r:id="Rf1bce98009d44393"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enlaces" sheetId="6" r:id="R76632472be594711"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="7" r:id="R58367158bad44ac3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido" sheetId="1" r:id="R48820b4b64444ac7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrusel" sheetId="2" r:id="Rd98dda2202234bf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investigación" sheetId="3" r:id="R92c9bff95ae8485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="4" r:id="Raab659a9e88d491f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="5" r:id="R921faeceef49411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enlaces" sheetId="6" r:id="R9ab1ad053ef74835"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="7" r:id="Rcc8e32627cf64696"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1469,7 +1469,7 @@
       </x:c>
       <x:c r="D54" s="10" t="str">
         <x:v>Av. Universidad 1001, Edificio 43
-Col. Chamilpa
+Col. Chamilpa, C.P. 62209
 Cuernavaca, Morelos, México</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
@@ -1639,7 +1639,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dfdf6a0e6784d63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R118b0ed6377f4d41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2275,7 +2275,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba27f917702e422b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd06f0de2ea064bda"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2851,7 +2851,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5ef5c12f2e4404c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9058d2f2471a486c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3383,7 +3383,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b1c9774ef6e476a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0ac98a046964460"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3997,7 +3997,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1190ffcad99f45ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85ce9783dfcc4264"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4497,7 +4497,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ca0325920714853"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa173667b4614b23"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Agregar apartado de liderazgo al equipo
</commit_message>
<xml_diff>
--- a/labsemco-contenido-google-sheets.xlsx
+++ b/labsemco-contenido-google-sheets.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido" sheetId="1" r:id="R48820b4b64444ac7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrusel" sheetId="2" r:id="Rd98dda2202234bf3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investigación" sheetId="3" r:id="R92c9bff95ae8485f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="4" r:id="Raab659a9e88d491f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="5" r:id="R921faeceef49411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enlaces" sheetId="6" r:id="R9ab1ad053ef74835"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="7" r:id="Rcc8e32627cf64696"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido" sheetId="1" r:id="Rac97394fa6a4413a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrusel" sheetId="2" r:id="R3da8207f48f541ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investigación" sheetId="3" r:id="R31eee3ab01b3457b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="4" r:id="R84848e03f6e340e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="5" r:id="Re41dcd1426bd4086"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enlaces" sheetId="6" r:id="R10ef597182fc406d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="7" r:id="Rc8bf6ecc4c0748e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1639,7 +1639,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R118b0ed6377f4d41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2291dd716ed2466f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2275,7 +2275,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd06f0de2ea064bda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ca9941dc94f424f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2851,7 +2851,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9058d2f2471a486c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75de4edc99dc446d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3383,7 +3383,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0ac98a046964460"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ce9cd127c0b4f91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3986,7 +3986,7 @@
       <x:c r="H101" s="17"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="G2:G101">
       <x:formula1>"SI,NO"</x:formula1>
     </x:dataValidation>
@@ -3994,10 +3994,13 @@
       <x:formula1>1</x:formula1>
       <x:formula2>999</x:formula2>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="B2:B101">
+      <x:formula1>"lider,colaboradores,estudiantes"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85ce9783dfcc4264"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86c2ad5a456743a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4497,7 +4500,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa173667b4614b23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3ab634a595d44fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4630,7 +4633,7 @@
         <x:v>Equipo</x:v>
       </x:c>
       <x:c r="B10" s="45" t="str">
-        <x:v>Cada fila crea una persona. Usa GRUPO: colaboradores o estudiantes.</x:v>
+        <x:v>Cada fila crea una persona. Usa GRUPO: lider, colaboradores o estudiantes.</x:v>
       </x:c>
       <x:c r="C10" s="45"/>
       <x:c r="D10" s="47" t="str">

</xml_diff>

<commit_message>
Permitir enlaces en tarjetas de proyectos
</commit_message>
<xml_diff>
--- a/labsemco-contenido-google-sheets.xlsx
+++ b/labsemco-contenido-google-sheets.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido" sheetId="1" r:id="Rac97394fa6a4413a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrusel" sheetId="2" r:id="R3da8207f48f541ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investigación" sheetId="3" r:id="R31eee3ab01b3457b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="4" r:id="R84848e03f6e340e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="5" r:id="Re41dcd1426bd4086"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enlaces" sheetId="6" r:id="R10ef597182fc406d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="7" r:id="Rc8bf6ecc4c0748e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido" sheetId="1" r:id="R982591e1924645a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrusel" sheetId="2" r:id="R24b4e676a6e740e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investigación" sheetId="3" r:id="R2fba96103c9b4308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="4" r:id="R629d1c0fd2214fa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="5" r:id="R834ffd9f9a9a47ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enlaces" sheetId="6" r:id="Rd462c30571d8487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="7" r:id="R48d2b9964bf548fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +22,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -64,8 +64,13 @@
       <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF26354A"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -90,6 +95,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFB0F1CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF006190"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFB9DFF0"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -122,7 +137,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="59">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -248,6 +263,24 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1639,7 +1672,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2291dd716ed2466f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fc785ee20ad4c35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2275,7 +2308,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ca9941dc94f424f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20de1d5108654c6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2851,7 +2884,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75de4edc99dc446d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8d665b0448a4667"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2870,6 +2903,8 @@
     <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2894,6 +2929,12 @@
       <x:c r="G1" s="9" t="str">
         <x:v>ORDEN</x:v>
       </x:c>
+      <x:c r="H1" s="54" t="str">
+        <x:v>ENLACE</x:v>
+      </x:c>
+      <x:c r="I1" s="54" t="str">
+        <x:v>TEXTO_ENLACE</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="10" t="str">
@@ -2917,6 +2958,8 @@
       <x:c r="G2" s="15" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="H2" s="58"/>
+      <x:c r="I2" s="58"/>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="10" t="str">
@@ -2940,6 +2983,8 @@
       <x:c r="G3" s="15" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="H3" s="57"/>
+      <x:c r="I3" s="57"/>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="10" t="str">
@@ -2963,6 +3008,8 @@
       <x:c r="G4" s="15" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="H4" s="58"/>
+      <x:c r="I4" s="58"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="11" t="str">
@@ -2986,390 +3033,584 @@
       <x:c r="G5" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="H5" s="57"/>
+      <x:c r="I5" s="57"/>
     </x:row>
     <x:row r="6">
       <x:c r="F6" s="14"/>
       <x:c r="G6" s="17"/>
+      <x:c r="H6" s="57"/>
+      <x:c r="I6" s="57"/>
     </x:row>
     <x:row r="7">
       <x:c r="F7" s="14"/>
       <x:c r="G7" s="17"/>
+      <x:c r="H7" s="57"/>
+      <x:c r="I7" s="57"/>
     </x:row>
     <x:row r="8">
       <x:c r="F8" s="14"/>
       <x:c r="G8" s="17"/>
+      <x:c r="H8" s="57"/>
+      <x:c r="I8" s="57"/>
     </x:row>
     <x:row r="9">
       <x:c r="F9" s="14"/>
       <x:c r="G9" s="17"/>
+      <x:c r="H9" s="57"/>
+      <x:c r="I9" s="57"/>
     </x:row>
     <x:row r="10">
       <x:c r="F10" s="14"/>
       <x:c r="G10" s="17"/>
+      <x:c r="H10" s="57"/>
+      <x:c r="I10" s="57"/>
     </x:row>
     <x:row r="11">
       <x:c r="F11" s="14"/>
       <x:c r="G11" s="17"/>
+      <x:c r="H11" s="57"/>
+      <x:c r="I11" s="57"/>
     </x:row>
     <x:row r="12">
       <x:c r="F12" s="14"/>
       <x:c r="G12" s="17"/>
+      <x:c r="H12" s="57"/>
+      <x:c r="I12" s="57"/>
     </x:row>
     <x:row r="13">
       <x:c r="F13" s="14"/>
       <x:c r="G13" s="17"/>
+      <x:c r="H13" s="57"/>
+      <x:c r="I13" s="57"/>
     </x:row>
     <x:row r="14">
       <x:c r="F14" s="14"/>
       <x:c r="G14" s="17"/>
+      <x:c r="H14" s="57"/>
+      <x:c r="I14" s="57"/>
     </x:row>
     <x:row r="15">
       <x:c r="F15" s="14"/>
       <x:c r="G15" s="17"/>
+      <x:c r="H15" s="57"/>
+      <x:c r="I15" s="57"/>
     </x:row>
     <x:row r="16">
       <x:c r="F16" s="14"/>
       <x:c r="G16" s="17"/>
+      <x:c r="H16" s="57"/>
+      <x:c r="I16" s="57"/>
     </x:row>
     <x:row r="17">
       <x:c r="F17" s="14"/>
       <x:c r="G17" s="17"/>
+      <x:c r="H17" s="57"/>
+      <x:c r="I17" s="57"/>
     </x:row>
     <x:row r="18">
       <x:c r="F18" s="14"/>
       <x:c r="G18" s="17"/>
+      <x:c r="H18" s="57"/>
+      <x:c r="I18" s="57"/>
     </x:row>
     <x:row r="19">
       <x:c r="F19" s="14"/>
       <x:c r="G19" s="17"/>
+      <x:c r="H19" s="57"/>
+      <x:c r="I19" s="57"/>
     </x:row>
     <x:row r="20">
       <x:c r="F20" s="14"/>
       <x:c r="G20" s="17"/>
+      <x:c r="H20" s="57"/>
+      <x:c r="I20" s="57"/>
     </x:row>
     <x:row r="21">
       <x:c r="F21" s="14"/>
       <x:c r="G21" s="17"/>
+      <x:c r="H21" s="57"/>
+      <x:c r="I21" s="57"/>
     </x:row>
     <x:row r="22">
       <x:c r="F22" s="14"/>
       <x:c r="G22" s="17"/>
+      <x:c r="H22" s="57"/>
+      <x:c r="I22" s="57"/>
     </x:row>
     <x:row r="23">
       <x:c r="F23" s="14"/>
       <x:c r="G23" s="17"/>
+      <x:c r="H23" s="57"/>
+      <x:c r="I23" s="57"/>
     </x:row>
     <x:row r="24">
       <x:c r="F24" s="14"/>
       <x:c r="G24" s="17"/>
+      <x:c r="H24" s="57"/>
+      <x:c r="I24" s="57"/>
     </x:row>
     <x:row r="25">
       <x:c r="F25" s="14"/>
       <x:c r="G25" s="17"/>
+      <x:c r="H25" s="57"/>
+      <x:c r="I25" s="57"/>
     </x:row>
     <x:row r="26">
       <x:c r="F26" s="14"/>
       <x:c r="G26" s="17"/>
+      <x:c r="H26" s="57"/>
+      <x:c r="I26" s="57"/>
     </x:row>
     <x:row r="27">
       <x:c r="F27" s="14"/>
       <x:c r="G27" s="17"/>
+      <x:c r="H27" s="57"/>
+      <x:c r="I27" s="57"/>
     </x:row>
     <x:row r="28">
       <x:c r="F28" s="14"/>
       <x:c r="G28" s="17"/>
+      <x:c r="H28" s="57"/>
+      <x:c r="I28" s="57"/>
     </x:row>
     <x:row r="29">
       <x:c r="F29" s="14"/>
       <x:c r="G29" s="17"/>
+      <x:c r="H29" s="57"/>
+      <x:c r="I29" s="57"/>
     </x:row>
     <x:row r="30">
       <x:c r="F30" s="14"/>
       <x:c r="G30" s="17"/>
+      <x:c r="H30" s="57"/>
+      <x:c r="I30" s="57"/>
     </x:row>
     <x:row r="31">
       <x:c r="F31" s="14"/>
       <x:c r="G31" s="17"/>
+      <x:c r="H31" s="57"/>
+      <x:c r="I31" s="57"/>
     </x:row>
     <x:row r="32">
       <x:c r="F32" s="14"/>
       <x:c r="G32" s="17"/>
+      <x:c r="H32" s="57"/>
+      <x:c r="I32" s="57"/>
     </x:row>
     <x:row r="33">
       <x:c r="F33" s="14"/>
       <x:c r="G33" s="17"/>
+      <x:c r="H33" s="57"/>
+      <x:c r="I33" s="57"/>
     </x:row>
     <x:row r="34">
       <x:c r="F34" s="14"/>
       <x:c r="G34" s="17"/>
+      <x:c r="H34" s="57"/>
+      <x:c r="I34" s="57"/>
     </x:row>
     <x:row r="35">
       <x:c r="F35" s="14"/>
       <x:c r="G35" s="17"/>
+      <x:c r="H35" s="57"/>
+      <x:c r="I35" s="57"/>
     </x:row>
     <x:row r="36">
       <x:c r="F36" s="14"/>
       <x:c r="G36" s="17"/>
+      <x:c r="H36" s="57"/>
+      <x:c r="I36" s="57"/>
     </x:row>
     <x:row r="37">
       <x:c r="F37" s="14"/>
       <x:c r="G37" s="17"/>
+      <x:c r="H37" s="57"/>
+      <x:c r="I37" s="57"/>
     </x:row>
     <x:row r="38">
       <x:c r="F38" s="14"/>
       <x:c r="G38" s="17"/>
+      <x:c r="H38" s="57"/>
+      <x:c r="I38" s="57"/>
     </x:row>
     <x:row r="39">
       <x:c r="F39" s="14"/>
       <x:c r="G39" s="17"/>
+      <x:c r="H39" s="57"/>
+      <x:c r="I39" s="57"/>
     </x:row>
     <x:row r="40">
       <x:c r="F40" s="14"/>
       <x:c r="G40" s="17"/>
+      <x:c r="H40" s="57"/>
+      <x:c r="I40" s="57"/>
     </x:row>
     <x:row r="41">
       <x:c r="F41" s="14"/>
       <x:c r="G41" s="17"/>
+      <x:c r="H41" s="57"/>
+      <x:c r="I41" s="57"/>
     </x:row>
     <x:row r="42">
       <x:c r="F42" s="14"/>
       <x:c r="G42" s="17"/>
+      <x:c r="H42" s="57"/>
+      <x:c r="I42" s="57"/>
     </x:row>
     <x:row r="43">
       <x:c r="F43" s="14"/>
       <x:c r="G43" s="17"/>
+      <x:c r="H43" s="57"/>
+      <x:c r="I43" s="57"/>
     </x:row>
     <x:row r="44">
       <x:c r="F44" s="14"/>
       <x:c r="G44" s="17"/>
+      <x:c r="H44" s="57"/>
+      <x:c r="I44" s="57"/>
     </x:row>
     <x:row r="45">
       <x:c r="F45" s="14"/>
       <x:c r="G45" s="17"/>
+      <x:c r="H45" s="57"/>
+      <x:c r="I45" s="57"/>
     </x:row>
     <x:row r="46">
       <x:c r="F46" s="14"/>
       <x:c r="G46" s="17"/>
+      <x:c r="H46" s="57"/>
+      <x:c r="I46" s="57"/>
     </x:row>
     <x:row r="47">
       <x:c r="F47" s="14"/>
       <x:c r="G47" s="17"/>
+      <x:c r="H47" s="57"/>
+      <x:c r="I47" s="57"/>
     </x:row>
     <x:row r="48">
       <x:c r="F48" s="14"/>
       <x:c r="G48" s="17"/>
+      <x:c r="H48" s="57"/>
+      <x:c r="I48" s="57"/>
     </x:row>
     <x:row r="49">
       <x:c r="F49" s="14"/>
       <x:c r="G49" s="17"/>
+      <x:c r="H49" s="57"/>
+      <x:c r="I49" s="57"/>
     </x:row>
     <x:row r="50">
       <x:c r="F50" s="14"/>
       <x:c r="G50" s="17"/>
+      <x:c r="H50" s="57"/>
+      <x:c r="I50" s="57"/>
     </x:row>
     <x:row r="51">
       <x:c r="F51" s="14"/>
       <x:c r="G51" s="17"/>
+      <x:c r="H51" s="57"/>
+      <x:c r="I51" s="57"/>
     </x:row>
     <x:row r="52">
       <x:c r="F52" s="14"/>
       <x:c r="G52" s="17"/>
+      <x:c r="H52" s="57"/>
+      <x:c r="I52" s="57"/>
     </x:row>
     <x:row r="53">
       <x:c r="F53" s="14"/>
       <x:c r="G53" s="17"/>
+      <x:c r="H53" s="57"/>
+      <x:c r="I53" s="57"/>
     </x:row>
     <x:row r="54">
       <x:c r="F54" s="14"/>
       <x:c r="G54" s="17"/>
+      <x:c r="H54" s="57"/>
+      <x:c r="I54" s="57"/>
     </x:row>
     <x:row r="55">
       <x:c r="F55" s="14"/>
       <x:c r="G55" s="17"/>
+      <x:c r="H55" s="57"/>
+      <x:c r="I55" s="57"/>
     </x:row>
     <x:row r="56">
       <x:c r="F56" s="14"/>
       <x:c r="G56" s="17"/>
+      <x:c r="H56" s="57"/>
+      <x:c r="I56" s="57"/>
     </x:row>
     <x:row r="57">
       <x:c r="F57" s="14"/>
       <x:c r="G57" s="17"/>
+      <x:c r="H57" s="57"/>
+      <x:c r="I57" s="57"/>
     </x:row>
     <x:row r="58">
       <x:c r="F58" s="14"/>
       <x:c r="G58" s="17"/>
+      <x:c r="H58" s="57"/>
+      <x:c r="I58" s="57"/>
     </x:row>
     <x:row r="59">
       <x:c r="F59" s="14"/>
       <x:c r="G59" s="17"/>
+      <x:c r="H59" s="57"/>
+      <x:c r="I59" s="57"/>
     </x:row>
     <x:row r="60">
       <x:c r="F60" s="14"/>
       <x:c r="G60" s="17"/>
+      <x:c r="H60" s="57"/>
+      <x:c r="I60" s="57"/>
     </x:row>
     <x:row r="61">
       <x:c r="F61" s="14"/>
       <x:c r="G61" s="17"/>
+      <x:c r="H61" s="57"/>
+      <x:c r="I61" s="57"/>
     </x:row>
     <x:row r="62">
       <x:c r="F62" s="14"/>
       <x:c r="G62" s="17"/>
+      <x:c r="H62" s="57"/>
+      <x:c r="I62" s="57"/>
     </x:row>
     <x:row r="63">
       <x:c r="F63" s="14"/>
       <x:c r="G63" s="17"/>
+      <x:c r="H63" s="57"/>
+      <x:c r="I63" s="57"/>
     </x:row>
     <x:row r="64">
       <x:c r="F64" s="14"/>
       <x:c r="G64" s="17"/>
+      <x:c r="H64" s="57"/>
+      <x:c r="I64" s="57"/>
     </x:row>
     <x:row r="65">
       <x:c r="F65" s="14"/>
       <x:c r="G65" s="17"/>
+      <x:c r="H65" s="57"/>
+      <x:c r="I65" s="57"/>
     </x:row>
     <x:row r="66">
       <x:c r="F66" s="14"/>
       <x:c r="G66" s="17"/>
+      <x:c r="H66" s="57"/>
+      <x:c r="I66" s="57"/>
     </x:row>
     <x:row r="67">
       <x:c r="F67" s="14"/>
       <x:c r="G67" s="17"/>
+      <x:c r="H67" s="57"/>
+      <x:c r="I67" s="57"/>
     </x:row>
     <x:row r="68">
       <x:c r="F68" s="14"/>
       <x:c r="G68" s="17"/>
+      <x:c r="H68" s="57"/>
+      <x:c r="I68" s="57"/>
     </x:row>
     <x:row r="69">
       <x:c r="F69" s="14"/>
       <x:c r="G69" s="17"/>
+      <x:c r="H69" s="57"/>
+      <x:c r="I69" s="57"/>
     </x:row>
     <x:row r="70">
       <x:c r="F70" s="14"/>
       <x:c r="G70" s="17"/>
+      <x:c r="H70" s="57"/>
+      <x:c r="I70" s="57"/>
     </x:row>
     <x:row r="71">
       <x:c r="F71" s="14"/>
       <x:c r="G71" s="17"/>
+      <x:c r="H71" s="57"/>
+      <x:c r="I71" s="57"/>
     </x:row>
     <x:row r="72">
       <x:c r="F72" s="14"/>
       <x:c r="G72" s="17"/>
+      <x:c r="H72" s="57"/>
+      <x:c r="I72" s="57"/>
     </x:row>
     <x:row r="73">
       <x:c r="F73" s="14"/>
       <x:c r="G73" s="17"/>
+      <x:c r="H73" s="57"/>
+      <x:c r="I73" s="57"/>
     </x:row>
     <x:row r="74">
       <x:c r="F74" s="14"/>
       <x:c r="G74" s="17"/>
+      <x:c r="H74" s="57"/>
+      <x:c r="I74" s="57"/>
     </x:row>
     <x:row r="75">
       <x:c r="F75" s="14"/>
       <x:c r="G75" s="17"/>
+      <x:c r="H75" s="57"/>
+      <x:c r="I75" s="57"/>
     </x:row>
     <x:row r="76">
       <x:c r="F76" s="14"/>
       <x:c r="G76" s="17"/>
+      <x:c r="H76" s="57"/>
+      <x:c r="I76" s="57"/>
     </x:row>
     <x:row r="77">
       <x:c r="F77" s="14"/>
       <x:c r="G77" s="17"/>
+      <x:c r="H77" s="57"/>
+      <x:c r="I77" s="57"/>
     </x:row>
     <x:row r="78">
       <x:c r="F78" s="14"/>
       <x:c r="G78" s="17"/>
+      <x:c r="H78" s="57"/>
+      <x:c r="I78" s="57"/>
     </x:row>
     <x:row r="79">
       <x:c r="F79" s="14"/>
       <x:c r="G79" s="17"/>
+      <x:c r="H79" s="57"/>
+      <x:c r="I79" s="57"/>
     </x:row>
     <x:row r="80">
       <x:c r="F80" s="14"/>
       <x:c r="G80" s="17"/>
+      <x:c r="H80" s="57"/>
+      <x:c r="I80" s="57"/>
     </x:row>
     <x:row r="81">
       <x:c r="F81" s="14"/>
       <x:c r="G81" s="17"/>
+      <x:c r="H81" s="57"/>
+      <x:c r="I81" s="57"/>
     </x:row>
     <x:row r="82">
       <x:c r="F82" s="14"/>
       <x:c r="G82" s="17"/>
+      <x:c r="H82" s="57"/>
+      <x:c r="I82" s="57"/>
     </x:row>
     <x:row r="83">
       <x:c r="F83" s="14"/>
       <x:c r="G83" s="17"/>
+      <x:c r="H83" s="57"/>
+      <x:c r="I83" s="57"/>
     </x:row>
     <x:row r="84">
       <x:c r="F84" s="14"/>
       <x:c r="G84" s="17"/>
+      <x:c r="H84" s="57"/>
+      <x:c r="I84" s="57"/>
     </x:row>
     <x:row r="85">
       <x:c r="F85" s="14"/>
       <x:c r="G85" s="17"/>
+      <x:c r="H85" s="57"/>
+      <x:c r="I85" s="57"/>
     </x:row>
     <x:row r="86">
       <x:c r="F86" s="14"/>
       <x:c r="G86" s="17"/>
+      <x:c r="H86" s="57"/>
+      <x:c r="I86" s="57"/>
     </x:row>
     <x:row r="87">
       <x:c r="F87" s="14"/>
       <x:c r="G87" s="17"/>
+      <x:c r="H87" s="57"/>
+      <x:c r="I87" s="57"/>
     </x:row>
     <x:row r="88">
       <x:c r="F88" s="14"/>
       <x:c r="G88" s="17"/>
+      <x:c r="H88" s="57"/>
+      <x:c r="I88" s="57"/>
     </x:row>
     <x:row r="89">
       <x:c r="F89" s="14"/>
       <x:c r="G89" s="17"/>
+      <x:c r="H89" s="57"/>
+      <x:c r="I89" s="57"/>
     </x:row>
     <x:row r="90">
       <x:c r="F90" s="14"/>
       <x:c r="G90" s="17"/>
+      <x:c r="H90" s="57"/>
+      <x:c r="I90" s="57"/>
     </x:row>
     <x:row r="91">
       <x:c r="F91" s="14"/>
       <x:c r="G91" s="17"/>
+      <x:c r="H91" s="57"/>
+      <x:c r="I91" s="57"/>
     </x:row>
     <x:row r="92">
       <x:c r="F92" s="14"/>
       <x:c r="G92" s="17"/>
+      <x:c r="H92" s="57"/>
+      <x:c r="I92" s="57"/>
     </x:row>
     <x:row r="93">
       <x:c r="F93" s="14"/>
       <x:c r="G93" s="17"/>
+      <x:c r="H93" s="57"/>
+      <x:c r="I93" s="57"/>
     </x:row>
     <x:row r="94">
       <x:c r="F94" s="14"/>
       <x:c r="G94" s="17"/>
+      <x:c r="H94" s="57"/>
+      <x:c r="I94" s="57"/>
     </x:row>
     <x:row r="95">
       <x:c r="F95" s="14"/>
       <x:c r="G95" s="17"/>
+      <x:c r="H95" s="57"/>
+      <x:c r="I95" s="57"/>
     </x:row>
     <x:row r="96">
       <x:c r="F96" s="14"/>
       <x:c r="G96" s="17"/>
+      <x:c r="H96" s="57"/>
+      <x:c r="I96" s="57"/>
     </x:row>
     <x:row r="97">
       <x:c r="F97" s="14"/>
       <x:c r="G97" s="17"/>
+      <x:c r="H97" s="57"/>
+      <x:c r="I97" s="57"/>
     </x:row>
     <x:row r="98">
       <x:c r="F98" s="14"/>
       <x:c r="G98" s="17"/>
+      <x:c r="H98" s="57"/>
+      <x:c r="I98" s="57"/>
     </x:row>
     <x:row r="99">
       <x:c r="F99" s="14"/>
       <x:c r="G99" s="17"/>
+      <x:c r="H99" s="57"/>
+      <x:c r="I99" s="57"/>
     </x:row>
     <x:row r="100">
       <x:c r="F100" s="14"/>
       <x:c r="G100" s="17"/>
+      <x:c r="H100" s="57"/>
+      <x:c r="I100" s="57"/>
     </x:row>
     <x:row r="101">
       <x:c r="F101" s="14"/>
       <x:c r="G101" s="17"/>
+      <x:c r="H101" s="57"/>
+      <x:c r="I101" s="57"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
@@ -3383,7 +3624,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ce9cd127c0b4f91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03c36b5eb30f4fdd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4000,7 +4241,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86c2ad5a456743a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53ddee7e206647f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4500,7 +4741,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3ab634a595d44fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd924852a3d924725"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4615,7 +4856,7 @@
         <x:v>Proyectos</x:v>
       </x:c>
       <x:c r="B9" s="45" t="str">
-        <x:v>Cada fila crea una tarjeta de proyecto.</x:v>
+        <x:v>Cada fila crea una tarjeta. ENLACE agrega el repositorio y TEXTO_ENLACE cambia el texto del botón.</x:v>
       </x:c>
       <x:c r="C9" s="45"/>
       <x:c r="D9" s="47" t="str">

</xml_diff>

<commit_message>
Crear directorio y perfiles dinamicos del equipo
</commit_message>
<xml_diff>
--- a/labsemco-contenido-google-sheets.xlsx
+++ b/labsemco-contenido-google-sheets.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido" sheetId="1" r:id="R982591e1924645a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrusel" sheetId="2" r:id="R24b4e676a6e740e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investigación" sheetId="3" r:id="R2fba96103c9b4308"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="4" r:id="R629d1c0fd2214fa5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="5" r:id="R834ffd9f9a9a47ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enlaces" sheetId="6" r:id="Rd462c30571d8487f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="7" r:id="R48d2b9964bf548fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenido" sheetId="1" r:id="R52e18008301345ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carrusel" sheetId="2" r:id="R76029216601f4cc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investigación" sheetId="3" r:id="R124211d93644480f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos" sheetId="4" r:id="Refdf000e254c4c93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipo" sheetId="5" r:id="R3a36c89c218140f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enlaces" sheetId="6" r:id="Rcc1bc7b6530241b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="7" r:id="R5907664bddb249fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -70,7 +70,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -107,6 +107,11 @@
         <x:fgColor rgb="FFB9DFF0"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF006190"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -137,7 +142,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="65">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -281,6 +286,20 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1672,7 +1691,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fc785ee20ad4c35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9d2f300f15a4bbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2308,7 +2327,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20de1d5108654c6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd93a8eb40bb148d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2884,7 +2903,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8d665b0448a4667"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd413f87e4b884501"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3624,7 +3643,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03c36b5eb30f4fdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b86b96841ee4960"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3644,6 +3663,13 @@
     <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="34" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="48" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="38" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -3671,6 +3697,27 @@
       <x:c r="H1" s="9" t="str">
         <x:v>ORDEN</x:v>
       </x:c>
+      <x:c r="I1" s="62" t="str">
+        <x:v>NIVEL_ROL</x:v>
+      </x:c>
+      <x:c r="J1" s="62" t="str">
+        <x:v>TEMA_INVESTIGACION</x:v>
+      </x:c>
+      <x:c r="K1" s="62" t="str">
+        <x:v>TITULO_INVESTIGACION</x:v>
+      </x:c>
+      <x:c r="L1" s="62" t="str">
+        <x:v>RESUMEN</x:v>
+      </x:c>
+      <x:c r="M1" s="62" t="str">
+        <x:v>CORREO</x:v>
+      </x:c>
+      <x:c r="N1" s="62" t="str">
+        <x:v>PUBLICACIONES</x:v>
+      </x:c>
+      <x:c r="O1" s="62" t="str">
+        <x:v>GOOGLE_SCHOLAR</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="10" t="str">
@@ -3697,6 +3744,13 @@
       <x:c r="H2" s="15" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="I2" s="64"/>
+      <x:c r="J2" s="64"/>
+      <x:c r="K2" s="64"/>
+      <x:c r="L2" s="64"/>
+      <x:c r="M2" s="64"/>
+      <x:c r="N2" s="64"/>
+      <x:c r="O2" s="64"/>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="10" t="str">
@@ -3723,6 +3777,13 @@
       <x:c r="H3" s="15" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="I3" s="64"/>
+      <x:c r="J3" s="64"/>
+      <x:c r="K3" s="64"/>
+      <x:c r="L3" s="64"/>
+      <x:c r="M3" s="64"/>
+      <x:c r="N3" s="64"/>
+      <x:c r="O3" s="64"/>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="10" t="str">
@@ -3749,6 +3810,13 @@
       <x:c r="H4" s="15" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="I4" s="64"/>
+      <x:c r="J4" s="64"/>
+      <x:c r="K4" s="64"/>
+      <x:c r="L4" s="64"/>
+      <x:c r="M4" s="64"/>
+      <x:c r="N4" s="64"/>
+      <x:c r="O4" s="64"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="10" t="str">
@@ -3775,6 +3843,13 @@
       <x:c r="H5" s="15" t="n">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="I5" s="64"/>
+      <x:c r="J5" s="64"/>
+      <x:c r="K5" s="64"/>
+      <x:c r="L5" s="64"/>
+      <x:c r="M5" s="64"/>
+      <x:c r="N5" s="64"/>
+      <x:c r="O5" s="64"/>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="10" t="str">
@@ -3801,6 +3876,13 @@
       <x:c r="H6" s="15" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="I6" s="64"/>
+      <x:c r="J6" s="64"/>
+      <x:c r="K6" s="64"/>
+      <x:c r="L6" s="64"/>
+      <x:c r="M6" s="64"/>
+      <x:c r="N6" s="64"/>
+      <x:c r="O6" s="64"/>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="10" t="str">
@@ -3827,6 +3909,13 @@
       <x:c r="H7" s="15" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="I7" s="64"/>
+      <x:c r="J7" s="64"/>
+      <x:c r="K7" s="64"/>
+      <x:c r="L7" s="64"/>
+      <x:c r="M7" s="64"/>
+      <x:c r="N7" s="64"/>
+      <x:c r="O7" s="64"/>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="11" t="str">
@@ -3853,381 +3942,1039 @@
       <x:c r="H8" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="I8" s="64"/>
+      <x:c r="J8" s="64"/>
+      <x:c r="K8" s="64"/>
+      <x:c r="L8" s="64"/>
+      <x:c r="M8" s="64"/>
+      <x:c r="N8" s="64"/>
+      <x:c r="O8" s="64"/>
     </x:row>
     <x:row r="9">
       <x:c r="G9" s="14"/>
       <x:c r="H9" s="17"/>
+      <x:c r="I9" s="64"/>
+      <x:c r="J9" s="64"/>
+      <x:c r="K9" s="64"/>
+      <x:c r="L9" s="64"/>
+      <x:c r="M9" s="64"/>
+      <x:c r="N9" s="64"/>
+      <x:c r="O9" s="64"/>
     </x:row>
     <x:row r="10">
       <x:c r="G10" s="14"/>
       <x:c r="H10" s="17"/>
+      <x:c r="I10" s="64"/>
+      <x:c r="J10" s="64"/>
+      <x:c r="K10" s="64"/>
+      <x:c r="L10" s="64"/>
+      <x:c r="M10" s="64"/>
+      <x:c r="N10" s="64"/>
+      <x:c r="O10" s="64"/>
     </x:row>
     <x:row r="11">
       <x:c r="G11" s="14"/>
       <x:c r="H11" s="17"/>
+      <x:c r="I11" s="64"/>
+      <x:c r="J11" s="64"/>
+      <x:c r="K11" s="64"/>
+      <x:c r="L11" s="64"/>
+      <x:c r="M11" s="64"/>
+      <x:c r="N11" s="64"/>
+      <x:c r="O11" s="64"/>
     </x:row>
     <x:row r="12">
       <x:c r="G12" s="14"/>
       <x:c r="H12" s="17"/>
+      <x:c r="I12" s="64"/>
+      <x:c r="J12" s="64"/>
+      <x:c r="K12" s="64"/>
+      <x:c r="L12" s="64"/>
+      <x:c r="M12" s="64"/>
+      <x:c r="N12" s="64"/>
+      <x:c r="O12" s="64"/>
     </x:row>
     <x:row r="13">
       <x:c r="G13" s="14"/>
       <x:c r="H13" s="17"/>
+      <x:c r="I13" s="64"/>
+      <x:c r="J13" s="64"/>
+      <x:c r="K13" s="64"/>
+      <x:c r="L13" s="64"/>
+      <x:c r="M13" s="64"/>
+      <x:c r="N13" s="64"/>
+      <x:c r="O13" s="64"/>
     </x:row>
     <x:row r="14">
       <x:c r="G14" s="14"/>
       <x:c r="H14" s="17"/>
+      <x:c r="I14" s="64"/>
+      <x:c r="J14" s="64"/>
+      <x:c r="K14" s="64"/>
+      <x:c r="L14" s="64"/>
+      <x:c r="M14" s="64"/>
+      <x:c r="N14" s="64"/>
+      <x:c r="O14" s="64"/>
     </x:row>
     <x:row r="15">
       <x:c r="G15" s="14"/>
       <x:c r="H15" s="17"/>
+      <x:c r="I15" s="64"/>
+      <x:c r="J15" s="64"/>
+      <x:c r="K15" s="64"/>
+      <x:c r="L15" s="64"/>
+      <x:c r="M15" s="64"/>
+      <x:c r="N15" s="64"/>
+      <x:c r="O15" s="64"/>
     </x:row>
     <x:row r="16">
       <x:c r="G16" s="14"/>
       <x:c r="H16" s="17"/>
+      <x:c r="I16" s="64"/>
+      <x:c r="J16" s="64"/>
+      <x:c r="K16" s="64"/>
+      <x:c r="L16" s="64"/>
+      <x:c r="M16" s="64"/>
+      <x:c r="N16" s="64"/>
+      <x:c r="O16" s="64"/>
     </x:row>
     <x:row r="17">
       <x:c r="G17" s="14"/>
       <x:c r="H17" s="17"/>
+      <x:c r="I17" s="64"/>
+      <x:c r="J17" s="64"/>
+      <x:c r="K17" s="64"/>
+      <x:c r="L17" s="64"/>
+      <x:c r="M17" s="64"/>
+      <x:c r="N17" s="64"/>
+      <x:c r="O17" s="64"/>
     </x:row>
     <x:row r="18">
       <x:c r="G18" s="14"/>
       <x:c r="H18" s="17"/>
+      <x:c r="I18" s="64"/>
+      <x:c r="J18" s="64"/>
+      <x:c r="K18" s="64"/>
+      <x:c r="L18" s="64"/>
+      <x:c r="M18" s="64"/>
+      <x:c r="N18" s="64"/>
+      <x:c r="O18" s="64"/>
     </x:row>
     <x:row r="19">
       <x:c r="G19" s="14"/>
       <x:c r="H19" s="17"/>
+      <x:c r="I19" s="64"/>
+      <x:c r="J19" s="64"/>
+      <x:c r="K19" s="64"/>
+      <x:c r="L19" s="64"/>
+      <x:c r="M19" s="64"/>
+      <x:c r="N19" s="64"/>
+      <x:c r="O19" s="64"/>
     </x:row>
     <x:row r="20">
       <x:c r="G20" s="14"/>
       <x:c r="H20" s="17"/>
+      <x:c r="I20" s="64"/>
+      <x:c r="J20" s="64"/>
+      <x:c r="K20" s="64"/>
+      <x:c r="L20" s="64"/>
+      <x:c r="M20" s="64"/>
+      <x:c r="N20" s="64"/>
+      <x:c r="O20" s="64"/>
     </x:row>
     <x:row r="21">
       <x:c r="G21" s="14"/>
       <x:c r="H21" s="17"/>
+      <x:c r="I21" s="64"/>
+      <x:c r="J21" s="64"/>
+      <x:c r="K21" s="64"/>
+      <x:c r="L21" s="64"/>
+      <x:c r="M21" s="64"/>
+      <x:c r="N21" s="64"/>
+      <x:c r="O21" s="64"/>
     </x:row>
     <x:row r="22">
       <x:c r="G22" s="14"/>
       <x:c r="H22" s="17"/>
+      <x:c r="I22" s="64"/>
+      <x:c r="J22" s="64"/>
+      <x:c r="K22" s="64"/>
+      <x:c r="L22" s="64"/>
+      <x:c r="M22" s="64"/>
+      <x:c r="N22" s="64"/>
+      <x:c r="O22" s="64"/>
     </x:row>
     <x:row r="23">
       <x:c r="G23" s="14"/>
       <x:c r="H23" s="17"/>
+      <x:c r="I23" s="64"/>
+      <x:c r="J23" s="64"/>
+      <x:c r="K23" s="64"/>
+      <x:c r="L23" s="64"/>
+      <x:c r="M23" s="64"/>
+      <x:c r="N23" s="64"/>
+      <x:c r="O23" s="64"/>
     </x:row>
     <x:row r="24">
       <x:c r="G24" s="14"/>
       <x:c r="H24" s="17"/>
+      <x:c r="I24" s="64"/>
+      <x:c r="J24" s="64"/>
+      <x:c r="K24" s="64"/>
+      <x:c r="L24" s="64"/>
+      <x:c r="M24" s="64"/>
+      <x:c r="N24" s="64"/>
+      <x:c r="O24" s="64"/>
     </x:row>
     <x:row r="25">
       <x:c r="G25" s="14"/>
       <x:c r="H25" s="17"/>
+      <x:c r="I25" s="64"/>
+      <x:c r="J25" s="64"/>
+      <x:c r="K25" s="64"/>
+      <x:c r="L25" s="64"/>
+      <x:c r="M25" s="64"/>
+      <x:c r="N25" s="64"/>
+      <x:c r="O25" s="64"/>
     </x:row>
     <x:row r="26">
       <x:c r="G26" s="14"/>
       <x:c r="H26" s="17"/>
+      <x:c r="I26" s="64"/>
+      <x:c r="J26" s="64"/>
+      <x:c r="K26" s="64"/>
+      <x:c r="L26" s="64"/>
+      <x:c r="M26" s="64"/>
+      <x:c r="N26" s="64"/>
+      <x:c r="O26" s="64"/>
     </x:row>
     <x:row r="27">
       <x:c r="G27" s="14"/>
       <x:c r="H27" s="17"/>
+      <x:c r="I27" s="64"/>
+      <x:c r="J27" s="64"/>
+      <x:c r="K27" s="64"/>
+      <x:c r="L27" s="64"/>
+      <x:c r="M27" s="64"/>
+      <x:c r="N27" s="64"/>
+      <x:c r="O27" s="64"/>
     </x:row>
     <x:row r="28">
       <x:c r="G28" s="14"/>
       <x:c r="H28" s="17"/>
+      <x:c r="I28" s="64"/>
+      <x:c r="J28" s="64"/>
+      <x:c r="K28" s="64"/>
+      <x:c r="L28" s="64"/>
+      <x:c r="M28" s="64"/>
+      <x:c r="N28" s="64"/>
+      <x:c r="O28" s="64"/>
     </x:row>
     <x:row r="29">
       <x:c r="G29" s="14"/>
       <x:c r="H29" s="17"/>
+      <x:c r="I29" s="64"/>
+      <x:c r="J29" s="64"/>
+      <x:c r="K29" s="64"/>
+      <x:c r="L29" s="64"/>
+      <x:c r="M29" s="64"/>
+      <x:c r="N29" s="64"/>
+      <x:c r="O29" s="64"/>
     </x:row>
     <x:row r="30">
       <x:c r="G30" s="14"/>
       <x:c r="H30" s="17"/>
+      <x:c r="I30" s="64"/>
+      <x:c r="J30" s="64"/>
+      <x:c r="K30" s="64"/>
+      <x:c r="L30" s="64"/>
+      <x:c r="M30" s="64"/>
+      <x:c r="N30" s="64"/>
+      <x:c r="O30" s="64"/>
     </x:row>
     <x:row r="31">
       <x:c r="G31" s="14"/>
       <x:c r="H31" s="17"/>
+      <x:c r="I31" s="64"/>
+      <x:c r="J31" s="64"/>
+      <x:c r="K31" s="64"/>
+      <x:c r="L31" s="64"/>
+      <x:c r="M31" s="64"/>
+      <x:c r="N31" s="64"/>
+      <x:c r="O31" s="64"/>
     </x:row>
     <x:row r="32">
       <x:c r="G32" s="14"/>
       <x:c r="H32" s="17"/>
+      <x:c r="I32" s="64"/>
+      <x:c r="J32" s="64"/>
+      <x:c r="K32" s="64"/>
+      <x:c r="L32" s="64"/>
+      <x:c r="M32" s="64"/>
+      <x:c r="N32" s="64"/>
+      <x:c r="O32" s="64"/>
     </x:row>
     <x:row r="33">
       <x:c r="G33" s="14"/>
       <x:c r="H33" s="17"/>
+      <x:c r="I33" s="64"/>
+      <x:c r="J33" s="64"/>
+      <x:c r="K33" s="64"/>
+      <x:c r="L33" s="64"/>
+      <x:c r="M33" s="64"/>
+      <x:c r="N33" s="64"/>
+      <x:c r="O33" s="64"/>
     </x:row>
     <x:row r="34">
       <x:c r="G34" s="14"/>
       <x:c r="H34" s="17"/>
+      <x:c r="I34" s="64"/>
+      <x:c r="J34" s="64"/>
+      <x:c r="K34" s="64"/>
+      <x:c r="L34" s="64"/>
+      <x:c r="M34" s="64"/>
+      <x:c r="N34" s="64"/>
+      <x:c r="O34" s="64"/>
     </x:row>
     <x:row r="35">
       <x:c r="G35" s="14"/>
       <x:c r="H35" s="17"/>
+      <x:c r="I35" s="64"/>
+      <x:c r="J35" s="64"/>
+      <x:c r="K35" s="64"/>
+      <x:c r="L35" s="64"/>
+      <x:c r="M35" s="64"/>
+      <x:c r="N35" s="64"/>
+      <x:c r="O35" s="64"/>
     </x:row>
     <x:row r="36">
       <x:c r="G36" s="14"/>
       <x:c r="H36" s="17"/>
+      <x:c r="I36" s="64"/>
+      <x:c r="J36" s="64"/>
+      <x:c r="K36" s="64"/>
+      <x:c r="L36" s="64"/>
+      <x:c r="M36" s="64"/>
+      <x:c r="N36" s="64"/>
+      <x:c r="O36" s="64"/>
     </x:row>
     <x:row r="37">
       <x:c r="G37" s="14"/>
       <x:c r="H37" s="17"/>
+      <x:c r="I37" s="64"/>
+      <x:c r="J37" s="64"/>
+      <x:c r="K37" s="64"/>
+      <x:c r="L37" s="64"/>
+      <x:c r="M37" s="64"/>
+      <x:c r="N37" s="64"/>
+      <x:c r="O37" s="64"/>
     </x:row>
     <x:row r="38">
       <x:c r="G38" s="14"/>
       <x:c r="H38" s="17"/>
+      <x:c r="I38" s="64"/>
+      <x:c r="J38" s="64"/>
+      <x:c r="K38" s="64"/>
+      <x:c r="L38" s="64"/>
+      <x:c r="M38" s="64"/>
+      <x:c r="N38" s="64"/>
+      <x:c r="O38" s="64"/>
     </x:row>
     <x:row r="39">
       <x:c r="G39" s="14"/>
       <x:c r="H39" s="17"/>
+      <x:c r="I39" s="64"/>
+      <x:c r="J39" s="64"/>
+      <x:c r="K39" s="64"/>
+      <x:c r="L39" s="64"/>
+      <x:c r="M39" s="64"/>
+      <x:c r="N39" s="64"/>
+      <x:c r="O39" s="64"/>
     </x:row>
     <x:row r="40">
       <x:c r="G40" s="14"/>
       <x:c r="H40" s="17"/>
+      <x:c r="I40" s="64"/>
+      <x:c r="J40" s="64"/>
+      <x:c r="K40" s="64"/>
+      <x:c r="L40" s="64"/>
+      <x:c r="M40" s="64"/>
+      <x:c r="N40" s="64"/>
+      <x:c r="O40" s="64"/>
     </x:row>
     <x:row r="41">
       <x:c r="G41" s="14"/>
       <x:c r="H41" s="17"/>
+      <x:c r="I41" s="64"/>
+      <x:c r="J41" s="64"/>
+      <x:c r="K41" s="64"/>
+      <x:c r="L41" s="64"/>
+      <x:c r="M41" s="64"/>
+      <x:c r="N41" s="64"/>
+      <x:c r="O41" s="64"/>
     </x:row>
     <x:row r="42">
       <x:c r="G42" s="14"/>
       <x:c r="H42" s="17"/>
+      <x:c r="I42" s="64"/>
+      <x:c r="J42" s="64"/>
+      <x:c r="K42" s="64"/>
+      <x:c r="L42" s="64"/>
+      <x:c r="M42" s="64"/>
+      <x:c r="N42" s="64"/>
+      <x:c r="O42" s="64"/>
     </x:row>
     <x:row r="43">
       <x:c r="G43" s="14"/>
       <x:c r="H43" s="17"/>
+      <x:c r="I43" s="64"/>
+      <x:c r="J43" s="64"/>
+      <x:c r="K43" s="64"/>
+      <x:c r="L43" s="64"/>
+      <x:c r="M43" s="64"/>
+      <x:c r="N43" s="64"/>
+      <x:c r="O43" s="64"/>
     </x:row>
     <x:row r="44">
       <x:c r="G44" s="14"/>
       <x:c r="H44" s="17"/>
+      <x:c r="I44" s="64"/>
+      <x:c r="J44" s="64"/>
+      <x:c r="K44" s="64"/>
+      <x:c r="L44" s="64"/>
+      <x:c r="M44" s="64"/>
+      <x:c r="N44" s="64"/>
+      <x:c r="O44" s="64"/>
     </x:row>
     <x:row r="45">
       <x:c r="G45" s="14"/>
       <x:c r="H45" s="17"/>
+      <x:c r="I45" s="64"/>
+      <x:c r="J45" s="64"/>
+      <x:c r="K45" s="64"/>
+      <x:c r="L45" s="64"/>
+      <x:c r="M45" s="64"/>
+      <x:c r="N45" s="64"/>
+      <x:c r="O45" s="64"/>
     </x:row>
     <x:row r="46">
       <x:c r="G46" s="14"/>
       <x:c r="H46" s="17"/>
+      <x:c r="I46" s="64"/>
+      <x:c r="J46" s="64"/>
+      <x:c r="K46" s="64"/>
+      <x:c r="L46" s="64"/>
+      <x:c r="M46" s="64"/>
+      <x:c r="N46" s="64"/>
+      <x:c r="O46" s="64"/>
     </x:row>
     <x:row r="47">
       <x:c r="G47" s="14"/>
       <x:c r="H47" s="17"/>
+      <x:c r="I47" s="64"/>
+      <x:c r="J47" s="64"/>
+      <x:c r="K47" s="64"/>
+      <x:c r="L47" s="64"/>
+      <x:c r="M47" s="64"/>
+      <x:c r="N47" s="64"/>
+      <x:c r="O47" s="64"/>
     </x:row>
     <x:row r="48">
       <x:c r="G48" s="14"/>
       <x:c r="H48" s="17"/>
+      <x:c r="I48" s="64"/>
+      <x:c r="J48" s="64"/>
+      <x:c r="K48" s="64"/>
+      <x:c r="L48" s="64"/>
+      <x:c r="M48" s="64"/>
+      <x:c r="N48" s="64"/>
+      <x:c r="O48" s="64"/>
     </x:row>
     <x:row r="49">
       <x:c r="G49" s="14"/>
       <x:c r="H49" s="17"/>
+      <x:c r="I49" s="64"/>
+      <x:c r="J49" s="64"/>
+      <x:c r="K49" s="64"/>
+      <x:c r="L49" s="64"/>
+      <x:c r="M49" s="64"/>
+      <x:c r="N49" s="64"/>
+      <x:c r="O49" s="64"/>
     </x:row>
     <x:row r="50">
       <x:c r="G50" s="14"/>
       <x:c r="H50" s="17"/>
+      <x:c r="I50" s="64"/>
+      <x:c r="J50" s="64"/>
+      <x:c r="K50" s="64"/>
+      <x:c r="L50" s="64"/>
+      <x:c r="M50" s="64"/>
+      <x:c r="N50" s="64"/>
+      <x:c r="O50" s="64"/>
     </x:row>
     <x:row r="51">
       <x:c r="G51" s="14"/>
       <x:c r="H51" s="17"/>
+      <x:c r="I51" s="64"/>
+      <x:c r="J51" s="64"/>
+      <x:c r="K51" s="64"/>
+      <x:c r="L51" s="64"/>
+      <x:c r="M51" s="64"/>
+      <x:c r="N51" s="64"/>
+      <x:c r="O51" s="64"/>
     </x:row>
     <x:row r="52">
       <x:c r="G52" s="14"/>
       <x:c r="H52" s="17"/>
+      <x:c r="I52" s="64"/>
+      <x:c r="J52" s="64"/>
+      <x:c r="K52" s="64"/>
+      <x:c r="L52" s="64"/>
+      <x:c r="M52" s="64"/>
+      <x:c r="N52" s="64"/>
+      <x:c r="O52" s="64"/>
     </x:row>
     <x:row r="53">
       <x:c r="G53" s="14"/>
       <x:c r="H53" s="17"/>
+      <x:c r="I53" s="64"/>
+      <x:c r="J53" s="64"/>
+      <x:c r="K53" s="64"/>
+      <x:c r="L53" s="64"/>
+      <x:c r="M53" s="64"/>
+      <x:c r="N53" s="64"/>
+      <x:c r="O53" s="64"/>
     </x:row>
     <x:row r="54">
       <x:c r="G54" s="14"/>
       <x:c r="H54" s="17"/>
+      <x:c r="I54" s="64"/>
+      <x:c r="J54" s="64"/>
+      <x:c r="K54" s="64"/>
+      <x:c r="L54" s="64"/>
+      <x:c r="M54" s="64"/>
+      <x:c r="N54" s="64"/>
+      <x:c r="O54" s="64"/>
     </x:row>
     <x:row r="55">
       <x:c r="G55" s="14"/>
       <x:c r="H55" s="17"/>
+      <x:c r="I55" s="64"/>
+      <x:c r="J55" s="64"/>
+      <x:c r="K55" s="64"/>
+      <x:c r="L55" s="64"/>
+      <x:c r="M55" s="64"/>
+      <x:c r="N55" s="64"/>
+      <x:c r="O55" s="64"/>
     </x:row>
     <x:row r="56">
       <x:c r="G56" s="14"/>
       <x:c r="H56" s="17"/>
+      <x:c r="I56" s="64"/>
+      <x:c r="J56" s="64"/>
+      <x:c r="K56" s="64"/>
+      <x:c r="L56" s="64"/>
+      <x:c r="M56" s="64"/>
+      <x:c r="N56" s="64"/>
+      <x:c r="O56" s="64"/>
     </x:row>
     <x:row r="57">
       <x:c r="G57" s="14"/>
       <x:c r="H57" s="17"/>
+      <x:c r="I57" s="64"/>
+      <x:c r="J57" s="64"/>
+      <x:c r="K57" s="64"/>
+      <x:c r="L57" s="64"/>
+      <x:c r="M57" s="64"/>
+      <x:c r="N57" s="64"/>
+      <x:c r="O57" s="64"/>
     </x:row>
     <x:row r="58">
       <x:c r="G58" s="14"/>
       <x:c r="H58" s="17"/>
+      <x:c r="I58" s="64"/>
+      <x:c r="J58" s="64"/>
+      <x:c r="K58" s="64"/>
+      <x:c r="L58" s="64"/>
+      <x:c r="M58" s="64"/>
+      <x:c r="N58" s="64"/>
+      <x:c r="O58" s="64"/>
     </x:row>
     <x:row r="59">
       <x:c r="G59" s="14"/>
       <x:c r="H59" s="17"/>
+      <x:c r="I59" s="64"/>
+      <x:c r="J59" s="64"/>
+      <x:c r="K59" s="64"/>
+      <x:c r="L59" s="64"/>
+      <x:c r="M59" s="64"/>
+      <x:c r="N59" s="64"/>
+      <x:c r="O59" s="64"/>
     </x:row>
     <x:row r="60">
       <x:c r="G60" s="14"/>
       <x:c r="H60" s="17"/>
+      <x:c r="I60" s="64"/>
+      <x:c r="J60" s="64"/>
+      <x:c r="K60" s="64"/>
+      <x:c r="L60" s="64"/>
+      <x:c r="M60" s="64"/>
+      <x:c r="N60" s="64"/>
+      <x:c r="O60" s="64"/>
     </x:row>
     <x:row r="61">
       <x:c r="G61" s="14"/>
       <x:c r="H61" s="17"/>
+      <x:c r="I61" s="64"/>
+      <x:c r="J61" s="64"/>
+      <x:c r="K61" s="64"/>
+      <x:c r="L61" s="64"/>
+      <x:c r="M61" s="64"/>
+      <x:c r="N61" s="64"/>
+      <x:c r="O61" s="64"/>
     </x:row>
     <x:row r="62">
       <x:c r="G62" s="14"/>
       <x:c r="H62" s="17"/>
+      <x:c r="I62" s="64"/>
+      <x:c r="J62" s="64"/>
+      <x:c r="K62" s="64"/>
+      <x:c r="L62" s="64"/>
+      <x:c r="M62" s="64"/>
+      <x:c r="N62" s="64"/>
+      <x:c r="O62" s="64"/>
     </x:row>
     <x:row r="63">
       <x:c r="G63" s="14"/>
       <x:c r="H63" s="17"/>
+      <x:c r="I63" s="64"/>
+      <x:c r="J63" s="64"/>
+      <x:c r="K63" s="64"/>
+      <x:c r="L63" s="64"/>
+      <x:c r="M63" s="64"/>
+      <x:c r="N63" s="64"/>
+      <x:c r="O63" s="64"/>
     </x:row>
     <x:row r="64">
       <x:c r="G64" s="14"/>
       <x:c r="H64" s="17"/>
+      <x:c r="I64" s="64"/>
+      <x:c r="J64" s="64"/>
+      <x:c r="K64" s="64"/>
+      <x:c r="L64" s="64"/>
+      <x:c r="M64" s="64"/>
+      <x:c r="N64" s="64"/>
+      <x:c r="O64" s="64"/>
     </x:row>
     <x:row r="65">
       <x:c r="G65" s="14"/>
       <x:c r="H65" s="17"/>
+      <x:c r="I65" s="64"/>
+      <x:c r="J65" s="64"/>
+      <x:c r="K65" s="64"/>
+      <x:c r="L65" s="64"/>
+      <x:c r="M65" s="64"/>
+      <x:c r="N65" s="64"/>
+      <x:c r="O65" s="64"/>
     </x:row>
     <x:row r="66">
       <x:c r="G66" s="14"/>
       <x:c r="H66" s="17"/>
+      <x:c r="I66" s="64"/>
+      <x:c r="J66" s="64"/>
+      <x:c r="K66" s="64"/>
+      <x:c r="L66" s="64"/>
+      <x:c r="M66" s="64"/>
+      <x:c r="N66" s="64"/>
+      <x:c r="O66" s="64"/>
     </x:row>
     <x:row r="67">
       <x:c r="G67" s="14"/>
       <x:c r="H67" s="17"/>
+      <x:c r="I67" s="64"/>
+      <x:c r="J67" s="64"/>
+      <x:c r="K67" s="64"/>
+      <x:c r="L67" s="64"/>
+      <x:c r="M67" s="64"/>
+      <x:c r="N67" s="64"/>
+      <x:c r="O67" s="64"/>
     </x:row>
     <x:row r="68">
       <x:c r="G68" s="14"/>
       <x:c r="H68" s="17"/>
+      <x:c r="I68" s="64"/>
+      <x:c r="J68" s="64"/>
+      <x:c r="K68" s="64"/>
+      <x:c r="L68" s="64"/>
+      <x:c r="M68" s="64"/>
+      <x:c r="N68" s="64"/>
+      <x:c r="O68" s="64"/>
     </x:row>
     <x:row r="69">
       <x:c r="G69" s="14"/>
       <x:c r="H69" s="17"/>
+      <x:c r="I69" s="64"/>
+      <x:c r="J69" s="64"/>
+      <x:c r="K69" s="64"/>
+      <x:c r="L69" s="64"/>
+      <x:c r="M69" s="64"/>
+      <x:c r="N69" s="64"/>
+      <x:c r="O69" s="64"/>
     </x:row>
     <x:row r="70">
       <x:c r="G70" s="14"/>
       <x:c r="H70" s="17"/>
+      <x:c r="I70" s="64"/>
+      <x:c r="J70" s="64"/>
+      <x:c r="K70" s="64"/>
+      <x:c r="L70" s="64"/>
+      <x:c r="M70" s="64"/>
+      <x:c r="N70" s="64"/>
+      <x:c r="O70" s="64"/>
     </x:row>
     <x:row r="71">
       <x:c r="G71" s="14"/>
       <x:c r="H71" s="17"/>
+      <x:c r="I71" s="64"/>
+      <x:c r="J71" s="64"/>
+      <x:c r="K71" s="64"/>
+      <x:c r="L71" s="64"/>
+      <x:c r="M71" s="64"/>
+      <x:c r="N71" s="64"/>
+      <x:c r="O71" s="64"/>
     </x:row>
     <x:row r="72">
       <x:c r="G72" s="14"/>
       <x:c r="H72" s="17"/>
+      <x:c r="I72" s="64"/>
+      <x:c r="J72" s="64"/>
+      <x:c r="K72" s="64"/>
+      <x:c r="L72" s="64"/>
+      <x:c r="M72" s="64"/>
+      <x:c r="N72" s="64"/>
+      <x:c r="O72" s="64"/>
     </x:row>
     <x:row r="73">
       <x:c r="G73" s="14"/>
       <x:c r="H73" s="17"/>
+      <x:c r="I73" s="64"/>
+      <x:c r="J73" s="64"/>
+      <x:c r="K73" s="64"/>
+      <x:c r="L73" s="64"/>
+      <x:c r="M73" s="64"/>
+      <x:c r="N73" s="64"/>
+      <x:c r="O73" s="64"/>
     </x:row>
     <x:row r="74">
       <x:c r="G74" s="14"/>
       <x:c r="H74" s="17"/>
+      <x:c r="I74" s="64"/>
+      <x:c r="J74" s="64"/>
+      <x:c r="K74" s="64"/>
+      <x:c r="L74" s="64"/>
+      <x:c r="M74" s="64"/>
+      <x:c r="N74" s="64"/>
+      <x:c r="O74" s="64"/>
     </x:row>
     <x:row r="75">
       <x:c r="G75" s="14"/>
       <x:c r="H75" s="17"/>
+      <x:c r="I75" s="64"/>
+      <x:c r="J75" s="64"/>
+      <x:c r="K75" s="64"/>
+      <x:c r="L75" s="64"/>
+      <x:c r="M75" s="64"/>
+      <x:c r="N75" s="64"/>
+      <x:c r="O75" s="64"/>
     </x:row>
     <x:row r="76">
       <x:c r="G76" s="14"/>
       <x:c r="H76" s="17"/>
+      <x:c r="I76" s="64"/>
+      <x:c r="J76" s="64"/>
+      <x:c r="K76" s="64"/>
+      <x:c r="L76" s="64"/>
+      <x:c r="M76" s="64"/>
+      <x:c r="N76" s="64"/>
+      <x:c r="O76" s="64"/>
     </x:row>
     <x:row r="77">
       <x:c r="G77" s="14"/>
       <x:c r="H77" s="17"/>
+      <x:c r="I77" s="64"/>
+      <x:c r="J77" s="64"/>
+      <x:c r="K77" s="64"/>
+      <x:c r="L77" s="64"/>
+      <x:c r="M77" s="64"/>
+      <x:c r="N77" s="64"/>
+      <x:c r="O77" s="64"/>
     </x:row>
     <x:row r="78">
       <x:c r="G78" s="14"/>
       <x:c r="H78" s="17"/>
+      <x:c r="I78" s="64"/>
+      <x:c r="J78" s="64"/>
+      <x:c r="K78" s="64"/>
+      <x:c r="L78" s="64"/>
+      <x:c r="M78" s="64"/>
+      <x:c r="N78" s="64"/>
+      <x:c r="O78" s="64"/>
     </x:row>
     <x:row r="79">
       <x:c r="G79" s="14"/>
       <x:c r="H79" s="17"/>
+      <x:c r="I79" s="64"/>
+      <x:c r="J79" s="64"/>
+      <x:c r="K79" s="64"/>
+      <x:c r="L79" s="64"/>
+      <x:c r="M79" s="64"/>
+      <x:c r="N79" s="64"/>
+      <x:c r="O79" s="64"/>
     </x:row>
     <x:row r="80">
       <x:c r="G80" s="14"/>
       <x:c r="H80" s="17"/>
+      <x:c r="I80" s="64"/>
+      <x:c r="J80" s="64"/>
+      <x:c r="K80" s="64"/>
+      <x:c r="L80" s="64"/>
+      <x:c r="M80" s="64"/>
+      <x:c r="N80" s="64"/>
+      <x:c r="O80" s="64"/>
     </x:row>
     <x:row r="81">
       <x:c r="G81" s="14"/>
       <x:c r="H81" s="17"/>
+      <x:c r="I81" s="64"/>
+      <x:c r="J81" s="64"/>
+      <x:c r="K81" s="64"/>
+      <x:c r="L81" s="64"/>
+      <x:c r="M81" s="64"/>
+      <x:c r="N81" s="64"/>
+      <x:c r="O81" s="64"/>
     </x:row>
     <x:row r="82">
       <x:c r="G82" s="14"/>
       <x:c r="H82" s="17"/>
+      <x:c r="I82" s="64"/>
+      <x:c r="J82" s="64"/>
+      <x:c r="K82" s="64"/>
+      <x:c r="L82" s="64"/>
+      <x:c r="M82" s="64"/>
+      <x:c r="N82" s="64"/>
+      <x:c r="O82" s="64"/>
     </x:row>
     <x:row r="83">
       <x:c r="G83" s="14"/>
       <x:c r="H83" s="17"/>
+      <x:c r="I83" s="64"/>
+      <x:c r="J83" s="64"/>
+      <x:c r="K83" s="64"/>
+      <x:c r="L83" s="64"/>
+      <x:c r="M83" s="64"/>
+      <x:c r="N83" s="64"/>
+      <x:c r="O83" s="64"/>
     </x:row>
     <x:row r="84">
       <x:c r="G84" s="14"/>
       <x:c r="H84" s="17"/>
+      <x:c r="I84" s="64"/>
+      <x:c r="J84" s="64"/>
+      <x:c r="K84" s="64"/>
+      <x:c r="L84" s="64"/>
+      <x:c r="M84" s="64"/>
+      <x:c r="N84" s="64"/>
+      <x:c r="O84" s="64"/>
     </x:row>
     <x:row r="85">
       <x:c r="G85" s="14"/>
       <x:c r="H85" s="17"/>
+      <x:c r="I85" s="64"/>
+      <x:c r="J85" s="64"/>
+      <x:c r="K85" s="64"/>
+      <x:c r="L85" s="64"/>
+      <x:c r="M85" s="64"/>
+      <x:c r="N85" s="64"/>
+      <x:c r="O85" s="64"/>
     </x:row>
     <x:row r="86">
       <x:c r="G86" s="14"/>
       <x:c r="H86" s="17"/>
+      <x:c r="I86" s="64"/>
+      <x:c r="J86" s="64"/>
+      <x:c r="K86" s="64"/>
+      <x:c r="L86" s="64"/>
+      <x:c r="M86" s="64"/>
+      <x:c r="N86" s="64"/>
+      <x:c r="O86" s="64"/>
     </x:row>
     <x:row r="87">
       <x:c r="G87" s="14"/>
       <x:c r="H87" s="17"/>
+      <x:c r="I87" s="64"/>
+      <x:c r="J87" s="64"/>
+      <x:c r="K87" s="64"/>
+      <x:c r="L87" s="64"/>
+      <x:c r="M87" s="64"/>
+      <x:c r="N87" s="64"/>
+      <x:c r="O87" s="64"/>
     </x:row>
     <x:row r="88">
       <x:c r="G88" s="14"/>
       <x:c r="H88" s="17"/>
+      <x:c r="I88" s="64"/>
+      <x:c r="J88" s="64"/>
+      <x:c r="K88" s="64"/>
+      <x:c r="L88" s="64"/>
+      <x:c r="M88" s="64"/>
+      <x:c r="N88" s="64"/>
+      <x:c r="O88" s="64"/>
     </x:row>
     <x:row r="89">
       <x:c r="G89" s="14"/>
       <x:c r="H89" s="17"/>
+      <x:c r="I89" s="64"/>
+      <x:c r="J89" s="64"/>
+      <x:c r="K89" s="64"/>
+      <x:c r="L89" s="64"/>
+      <x:c r="M89" s="64"/>
+      <x:c r="N89" s="64"/>
+      <x:c r="O89" s="64"/>
     </x:row>
     <x:row r="90">
       <x:c r="G90" s="14"/>
       <x:c r="H90" s="17"/>
+      <x:c r="I90" s="64"/>
+      <x:c r="J90" s="64"/>
+      <x:c r="K90" s="64"/>
+      <x:c r="L90" s="64"/>
+      <x:c r="M90" s="64"/>
+      <x:c r="N90" s="64"/>
+      <x:c r="O90" s="64"/>
     </x:row>
     <x:row r="91">
       <x:c r="G91" s="14"/>
       <x:c r="H91" s="17"/>
+      <x:c r="I91" s="64"/>
+      <x:c r="J91" s="64"/>
+      <x:c r="K91" s="64"/>
+      <x:c r="L91" s="64"/>
+      <x:c r="M91" s="64"/>
+      <x:c r="N91" s="64"/>
+      <x:c r="O91" s="64"/>
     </x:row>
     <x:row r="92">
       <x:c r="G92" s="14"/>
       <x:c r="H92" s="17"/>
+      <x:c r="I92" s="64"/>
+      <x:c r="J92" s="64"/>
+      <x:c r="K92" s="64"/>
+      <x:c r="L92" s="64"/>
+      <x:c r="M92" s="64"/>
+      <x:c r="N92" s="64"/>
+      <x:c r="O92" s="64"/>
     </x:row>
     <x:row r="93">
       <x:c r="G93" s="14"/>
       <x:c r="H93" s="17"/>
+      <x:c r="I93" s="64"/>
+      <x:c r="J93" s="64"/>
+      <x:c r="K93" s="64"/>
+      <x:c r="L93" s="64"/>
+      <x:c r="M93" s="64"/>
+      <x:c r="N93" s="64"/>
+      <x:c r="O93" s="64"/>
     </x:row>
     <x:row r="94">
       <x:c r="G94" s="14"/>
       <x:c r="H94" s="17"/>
+      <x:c r="I94" s="64"/>
+      <x:c r="J94" s="64"/>
+      <x:c r="K94" s="64"/>
+      <x:c r="L94" s="64"/>
+      <x:c r="M94" s="64"/>
+      <x:c r="N94" s="64"/>
+      <x:c r="O94" s="64"/>
     </x:row>
     <x:row r="95">
       <x:c r="G95" s="14"/>
       <x:c r="H95" s="17"/>
+      <x:c r="I95" s="64"/>
+      <x:c r="J95" s="64"/>
+      <x:c r="K95" s="64"/>
+      <x:c r="L95" s="64"/>
+      <x:c r="M95" s="64"/>
+      <x:c r="N95" s="64"/>
+      <x:c r="O95" s="64"/>
     </x:row>
     <x:row r="96">
       <x:c r="G96" s="14"/>
       <x:c r="H96" s="17"/>
+      <x:c r="I96" s="64"/>
+      <x:c r="J96" s="64"/>
+      <x:c r="K96" s="64"/>
+      <x:c r="L96" s="64"/>
+      <x:c r="M96" s="64"/>
+      <x:c r="N96" s="64"/>
+      <x:c r="O96" s="64"/>
     </x:row>
     <x:row r="97">
       <x:c r="G97" s="14"/>
       <x:c r="H97" s="17"/>
+      <x:c r="I97" s="64"/>
+      <x:c r="J97" s="64"/>
+      <x:c r="K97" s="64"/>
+      <x:c r="L97" s="64"/>
+      <x:c r="M97" s="64"/>
+      <x:c r="N97" s="64"/>
+      <x:c r="O97" s="64"/>
     </x:row>
     <x:row r="98">
       <x:c r="G98" s="14"/>
       <x:c r="H98" s="17"/>
+      <x:c r="I98" s="64"/>
+      <x:c r="J98" s="64"/>
+      <x:c r="K98" s="64"/>
+      <x:c r="L98" s="64"/>
+      <x:c r="M98" s="64"/>
+      <x:c r="N98" s="64"/>
+      <x:c r="O98" s="64"/>
     </x:row>
     <x:row r="99">
       <x:c r="G99" s="14"/>
       <x:c r="H99" s="17"/>
+      <x:c r="I99" s="64"/>
+      <x:c r="J99" s="64"/>
+      <x:c r="K99" s="64"/>
+      <x:c r="L99" s="64"/>
+      <x:c r="M99" s="64"/>
+      <x:c r="N99" s="64"/>
+      <x:c r="O99" s="64"/>
     </x:row>
     <x:row r="100">
       <x:c r="G100" s="14"/>
       <x:c r="H100" s="17"/>
+      <x:c r="I100" s="64"/>
+      <x:c r="J100" s="64"/>
+      <x:c r="K100" s="64"/>
+      <x:c r="L100" s="64"/>
+      <x:c r="M100" s="64"/>
+      <x:c r="N100" s="64"/>
+      <x:c r="O100" s="64"/>
     </x:row>
     <x:row r="101">
       <x:c r="G101" s="14"/>
       <x:c r="H101" s="17"/>
+      <x:c r="I101" s="64"/>
+      <x:c r="J101" s="64"/>
+      <x:c r="K101" s="64"/>
+      <x:c r="L101" s="64"/>
+      <x:c r="M101" s="64"/>
+      <x:c r="N101" s="64"/>
+      <x:c r="O101" s="64"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="3">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="G2:G101">
       <x:formula1>"SI,NO"</x:formula1>
     </x:dataValidation>
@@ -4235,13 +4982,10 @@
       <x:formula1>1</x:formula1>
       <x:formula2>999</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="B2:B101">
-      <x:formula1>"lider,colaboradores,estudiantes"</x:formula1>
-    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53ddee7e206647f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3791e37ead0b40d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4741,7 +5485,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd924852a3d924725"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra722b03894c74352"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4874,7 +5618,7 @@
         <x:v>Equipo</x:v>
       </x:c>
       <x:c r="B10" s="45" t="str">
-        <x:v>Cada fila crea una persona. Usa GRUPO: lider, colaboradores o estudiantes.</x:v>
+        <x:v>Cada fila crea una ficha. GRUPO acepta cualquier categoría. Completa las columnas I:O para tema, nivel/rol, investigación, resumen, correo y publicaciones.</x:v>
       </x:c>
       <x:c r="C10" s="45"/>
       <x:c r="D10" s="47" t="str">

</xml_diff>